<commit_message>
Agregar formato profesional al reporte de motores
</commit_message>
<xml_diff>
--- a/resultados/motores_calculados.xlsx
+++ b/resultados/motores_calculados.xlsx
@@ -7,9 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="MOTORES" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RESUMEN" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MOTORES'!$A$1:$N$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RESUMEN'!$A$1:$B$10</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,16 +32,35 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -51,14 +74,52 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -427,236 +488,374 @@
   </sheetPr>
   <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>TAG</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>DESCRIPCION</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>HP</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>VOLTAJE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>FP</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>EFICIENCIA</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>CORRIENTE_PLACA_A</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>CORRIENTE_MEDIDA_A</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>ESTADO</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>KW</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>CORRIENTE_CALCULADA_A</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>DESVIACION_CALC_PLACA_PCT</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>CARGA_CORRIENTE_PCT</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>ALERTA</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>M-001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Bomba de agua</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="5" t="n">
         <v>125</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="5" t="n">
         <v>480</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="5" t="n">
         <v>0.88</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="5" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="5" t="n">
         <v>140</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="5" t="n">
         <v>120</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Operando</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="5" t="n">
         <v>93.25</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="5" t="n">
         <v>135.59</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="5" t="n">
         <v>-3.15</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" s="5" t="n">
         <v>85.70999999999999</v>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="6" t="inlineStr">
         <is>
           <t>NORMAL</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>M-002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Ventilador</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="5" t="n">
         <v>75</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="5" t="n">
         <v>480</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="5" t="n">
         <v>0.93</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="5" t="n">
         <v>82</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="5" t="n">
         <v>76</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Operando</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="5" t="n">
         <v>55.95</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="5" t="n">
         <v>80.40000000000001</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L3" s="5" t="n">
         <v>-1.95</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" s="5" t="n">
         <v>92.68000000000001</v>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N3" s="7" t="inlineStr">
         <is>
           <t>CARGA ALTA</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>M-003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Bomba condensado</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="5" t="n">
         <v>480</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="5" t="n">
         <v>0.87</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="5" t="n">
         <v>0.91</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="5" t="n">
         <v>32</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Operando</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="5" t="n">
         <v>22.38</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="5" t="n">
         <v>34</v>
       </c>
-      <c r="L4" t="n">
+      <c r="L4" s="5" t="n">
         <v>-2.85</v>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" s="5" t="n">
         <v>91.43000000000001</v>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N4" s="7" t="inlineStr">
         <is>
           <t>CARGA ALTA</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:N4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>INDICADOR</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>VALOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Total de motores</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Potencia instalada HP</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Potencia instalada kW</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>171.58</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Motores normales</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Motores con carga alta</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Motores con carga baja</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Motores con posible sobrecarga</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Corriente calculada total A</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>249.99</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Corriente medida total A</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>228</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Separar parametros de analisis de motores
</commit_message>
<xml_diff>
--- a/resultados/motores_calculados.xlsx
+++ b/resultados/motores_calculados.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MOTORES'!$A$1:$N$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RESUMEN'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RESUMEN'!$A$1:$B$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -854,8 +854,38 @@
         <v>228</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Límite carga baja %</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Límite carga alta %</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Límite sobrecarga %</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Integrar diagnostico trifasico al reporte de motores
</commit_message>
<xml_diff>
--- a/resultados/motores_calculados.xlsx
+++ b/resultados/motores_calculados.xlsx
@@ -11,8 +11,8 @@
     <sheet name="RESUMEN" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MOTORES'!$A$1:$N$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RESUMEN'!$A$1:$B$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MOTORES'!$A$1:$AB$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RESUMEN'!$A$1:$B$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,7 +37,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +57,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -101,25 +106,22 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -486,23 +488,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:AB4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="23" customWidth="1" min="18" max="18"/>
+    <col width="27" customWidth="1" min="19" max="19"/>
+    <col width="23" customWidth="1" min="20" max="20"/>
+    <col width="23" customWidth="1" min="21" max="21"/>
+    <col width="21" customWidth="1" min="22" max="22"/>
+    <col width="25" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="25" max="25"/>
+    <col width="30" customWidth="1" min="26" max="26"/>
+    <col width="28" customWidth="1" min="27" max="27"/>
+    <col width="42" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="45" customHeight="1">
@@ -543,37 +559,107 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>CORRIENTE_MEDIDA_A</t>
+          <t>CORRIENTE_L1_A</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
+          <t>CORRIENTE_L2_A</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>CORRIENTE_L3_A</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>VOLTAJE_L1_L2_V</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>VOLTAJE_L2_L3_V</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>VOLTAJE_L3_L1_V</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
           <t>ESTADO</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>KW</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>CORRIENTE_CALCULADA_A</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>DESVIACION_CALC_PLACA_PCT</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>CORRIENTE_PROMEDIO_A</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>DESBALANCE_CORRIENTE_PCT</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>FASE_MAYOR_CORRIENTE</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>FASE_MENOR_CORRIENTE</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>VOLTAJE_PROMEDIO_V</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>DESBALANCE_VOLTAJE_PCT</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>CARGA_CORRIENTE_PCT</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>ALERTA</t>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>ALERTA_CARGA</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>ALERTA_DESBALANCE_CORRIENTE</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>ALERTA_DESBALANCE_VOLTAJE</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>DIAGNOSTICO_GENERAL</t>
         </is>
       </c>
     </row>
@@ -583,47 +669,99 @@
           <t>M-001</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Bomba de agua</t>
         </is>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="4" t="n">
         <v>125</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="4" t="n">
         <v>480</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="E2" s="4" t="n">
         <v>0.88</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="4" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="G2" s="4" t="n">
         <v>140</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="4" t="n">
+        <v>118</v>
+      </c>
+      <c r="I2" s="4" t="n">
         <v>120</v>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="4" t="n">
+        <v>123</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>478</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>481</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>479</v>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Operando</t>
         </is>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="O2" s="4" t="n">
         <v>93.25</v>
       </c>
-      <c r="K2" s="5" t="n">
+      <c r="P2" s="4" t="n">
         <v>135.59</v>
       </c>
-      <c r="L2" s="5" t="n">
+      <c r="Q2" s="4" t="n">
         <v>-3.15</v>
       </c>
-      <c r="M2" s="5" t="n">
-        <v>85.70999999999999</v>
-      </c>
-      <c r="N2" s="6" t="inlineStr">
+      <c r="R2" s="4" t="n">
+        <v>120.33</v>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="U2" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="V2" s="4" t="n">
+        <v>479.33</v>
+      </c>
+      <c r="W2" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>85.95</v>
+      </c>
+      <c r="Y2" s="5" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="Z2" s="5" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="AA2" s="5" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="AB2" s="5" t="inlineStr">
         <is>
           <t>NORMAL</t>
         </is>
@@ -635,47 +773,99 @@
           <t>M-002</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Ventilador</t>
         </is>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="4" t="n">
         <v>480</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E3" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="4" t="n">
         <v>0.93</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="G3" s="4" t="n">
         <v>82</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="H3" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="I3" s="4" t="n">
         <v>76</v>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>477</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>480</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>482</v>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Operando</t>
         </is>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="O3" s="4" t="n">
         <v>55.95</v>
       </c>
-      <c r="K3" s="5" t="n">
+      <c r="P3" s="4" t="n">
         <v>80.40000000000001</v>
       </c>
-      <c r="L3" s="5" t="n">
+      <c r="Q3" s="4" t="n">
         <v>-1.95</v>
       </c>
-      <c r="M3" s="5" t="n">
-        <v>92.68000000000001</v>
-      </c>
-      <c r="N3" s="7" t="inlineStr">
+      <c r="R3" s="4" t="n">
+        <v>76.33</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="V3" s="4" t="n">
+        <v>479.67</v>
+      </c>
+      <c r="W3" s="4" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="X3" s="4" t="n">
+        <v>93.09</v>
+      </c>
+      <c r="Y3" s="6" t="inlineStr">
+        <is>
+          <t>CARGA ALTA</t>
+        </is>
+      </c>
+      <c r="Z3" s="5" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="AB3" s="7" t="inlineStr">
         <is>
           <t>CARGA ALTA</t>
         </is>
@@ -687,54 +877,106 @@
           <t>M-003</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Bomba condensado</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="4" t="n">
         <v>480</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="4" t="n">
         <v>0.87</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="4" t="n">
         <v>0.91</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="G4" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="H4" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="I4" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>479</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>478</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>481</v>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Operando</t>
         </is>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="O4" s="4" t="n">
         <v>22.38</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="P4" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="Q4" s="4" t="n">
         <v>-2.85</v>
       </c>
-      <c r="M4" s="5" t="n">
+      <c r="R4" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="n">
+        <v>479.33</v>
+      </c>
+      <c r="W4" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="X4" s="4" t="n">
         <v>91.43000000000001</v>
       </c>
-      <c r="N4" s="7" t="inlineStr">
+      <c r="Y4" s="6" t="inlineStr">
         <is>
           <t>CARGA ALTA</t>
         </is>
       </c>
+      <c r="Z4" s="5" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="AB4" s="7" t="inlineStr">
+        <is>
+          <t>CARGA ALTA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N4"/>
+  <autoFilter ref="A1:AB4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -745,11 +987,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -765,127 +1007,177 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Total de motores</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n">
+      <c r="B2" s="4" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Potencia instalada HP</t>
         </is>
       </c>
-      <c r="B3" s="9" t="n">
+      <c r="B3" s="4" t="n">
         <v>230</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Potencia instalada kW</t>
         </is>
       </c>
-      <c r="B4" s="9" t="n">
+      <c r="B4" s="4" t="n">
         <v>171.58</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Motores normales</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="n">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Motores diagnóstico normal</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Motores con carga alta</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Motores con carga baja</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Motores con posible sobrecarga</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Corriente calculada total A</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n">
-        <v>249.99</v>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Motores con desbalance de corriente</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Corriente medida total A</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="n">
-        <v>228</v>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Motores con desbalance de voltaje</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Mayor desbalance de corriente %</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>3.49</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Mayor desbalance de voltaje %</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Carga promedio por corriente %</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>90.16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Límite carga baja %</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B14" s="4" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Límite carga alta %</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B15" s="4" t="n">
         <v>90</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Límite sobrecarga %</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B16" s="4" t="n">
         <v>100</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Límite desbalance corriente %</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Límite desbalance voltaje %</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B13"/>
+  <autoFilter ref="A1:B18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Completar arquitectura modular del analisis de motores
</commit_message>
<xml_diff>
--- a/resultados/motores_calculados.xlsx
+++ b/resultados/motores_calculados.xlsx
@@ -37,7 +37,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -57,11 +57,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -117,12 +112,11 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -865,7 +859,7 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="AB3" s="7" t="inlineStr">
+      <c r="AB3" s="6" t="inlineStr">
         <is>
           <t>CARGA ALTA</t>
         </is>
@@ -969,7 +963,7 @@
           <t>NORMAL</t>
         </is>
       </c>
-      <c r="AB4" s="7" t="inlineStr">
+      <c r="AB4" s="6" t="inlineStr">
         <is>
           <t>CARGA ALTA</t>
         </is>
@@ -994,185 +988,185 @@
     <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>INDICADOR</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>VALOR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Total de motores</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="9" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Potencia instalada HP</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="9" t="n">
         <v>230</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Potencia instalada kW</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="9" t="n">
         <v>171.58</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Motores diagnóstico normal</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="9" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Motores con carga alta</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="9" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Motores con carga baja</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Motores con posible sobrecarga</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Motores con desbalance de corriente</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Motores con desbalance de voltaje</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Mayor desbalance de corriente %</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="9" t="n">
         <v>3.49</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Mayor desbalance de voltaje %</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="9" t="n">
         <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Carga promedio por corriente %</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="9" t="n">
         <v>90.16</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Límite carga baja %</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="9" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Límite carga alta %</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="9" t="n">
         <v>90</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Límite sobrecarga %</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B16" s="9" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Límite desbalance corriente %</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n">
+      <c r="B17" s="9" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Límite desbalance voltaje %</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n">
+      <c r="B18" s="9" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>